<commit_message>
updated data for inverts
</commit_message>
<xml_diff>
--- a/Invert_Core_Samples_fall_2025_Deborah.xlsx
+++ b/Invert_Core_Samples_fall_2025_Deborah.xlsx
@@ -8,16 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\011488124.CAMPUS-DOMAIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D5B594-07FB-4EBB-AD86-1D4562D6178D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067AB79D-2022-4C85-A3AE-07C77201F79B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{CC5B1F45-5237-4F41-9860-D6392839C0C3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{CC5B1F45-5237-4F41-9860-D6392839C0C3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Primer" sheetId="2" r:id="rId2"/>
-    <sheet name="Primer_Abundance" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId2"/>
+    <sheet name="Primer" sheetId="2" r:id="rId3"/>
+    <sheet name="Primer_Abundance" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="2" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="171">
   <si>
     <t>Species</t>
   </si>
@@ -543,6 +547,15 @@
   </si>
   <si>
     <t>Oribatida</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Count of Species</t>
   </si>
 </sst>
 </file>
@@ -618,7 +631,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -626,6 +639,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3669,6 +3687,1459 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Anita Arenas" refreshedDate="46226.466734490743" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="41" xr:uid="{F46002BD-9C36-4AB8-8EB1-D13F6ACE8996}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A5:Y45" sheet="Data"/>
+  </cacheSource>
+  <cacheFields count="25">
+    <cacheField name="Species" numFmtId="0">
+      <sharedItems count="38">
+        <s v="Tubificidae"/>
+        <s v="Enchytraeidae"/>
+        <s v="Pseudopolydora paucibranchiata"/>
+        <s v="Exogone Sp."/>
+        <s v="Capitella Sp."/>
+        <s v="Nereididae"/>
+        <s v="Fabricia Stellaris"/>
+        <s v="Gammaridae a"/>
+        <s v="Monocorophium"/>
+        <s v="Leptochelia dubia"/>
+        <s v="Phoronids"/>
+        <s v="Staphylinidae (rove)"/>
+        <s v="Polydora ligni"/>
+        <s v="Polydora nuchalis"/>
+        <s v="Streblospio benedicti"/>
+        <s v="Eteone sp"/>
+        <s v="Dolichopodidae"/>
+        <s v="Sea Anenome"/>
+        <s v="Flatworms"/>
+        <s v="Brania Sp"/>
+        <s v="Orbiniidae"/>
+        <s v="Grandidierella japonica"/>
+        <s v="Caprellids"/>
+        <s v="Capitellidae"/>
+        <s v="Assiminea californica"/>
+        <s v="Acteocina Sp"/>
+        <s v="A. lindahli"/>
+        <s v="Poduridae"/>
+        <s v="white mite"/>
+        <s v="brown mite"/>
+        <s v="Chrysopidae larva"/>
+        <s v="Acentrogobius nebulosus"/>
+        <s v="Exogone lourei"/>
+        <s v="Mediomastus acutus"/>
+        <s v="Eunicidae"/>
+        <s v="Mediomastus"/>
+        <s v="Tharyx sp."/>
+        <s v="Oribatida"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="UNBS3" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="32"/>
+    </cacheField>
+    <cacheField name="MALS1" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="MALS3" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="MALS12" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="3" maxValue="3"/>
+    </cacheField>
+    <cacheField name="MALS32" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="UNBS2" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="18"/>
+    </cacheField>
+    <cacheField name="UNBS1" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="15"/>
+    </cacheField>
+    <cacheField name="UNBS32" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="4"/>
+    </cacheField>
+    <cacheField name="UNBS4" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="5"/>
+    </cacheField>
+    <cacheField name="UNBS12" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="161"/>
+    </cacheField>
+    <cacheField name="UNBS42" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="10"/>
+    </cacheField>
+    <cacheField name="BOLS1" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="GOLS1" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="BOLS3" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="28"/>
+    </cacheField>
+    <cacheField name="MALS2" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="GOLS12" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="7"/>
+    </cacheField>
+    <cacheField name="VENS1" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="1"/>
+    </cacheField>
+    <cacheField name="GOLS2" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="BCS3" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="34"/>
+    </cacheField>
+    <cacheField name="BCS2" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="7" maxValue="24"/>
+    </cacheField>
+    <cacheField name="GOLS3" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="1"/>
+    </cacheField>
+    <cacheField name="SBNWRS1" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="2"/>
+    </cacheField>
+    <cacheField name="SBNWRS2" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="BCS1" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="4"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="41">
+  <r>
+    <x v="0"/>
+    <n v="31"/>
+    <m/>
+    <m/>
+    <n v="3"/>
+    <m/>
+    <n v="6"/>
+    <m/>
+    <n v="3"/>
+    <m/>
+    <n v="161"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="32"/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="32"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="18"/>
+    <n v="3"/>
+    <m/>
+    <m/>
+    <n v="29"/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <n v="7"/>
+    <m/>
+    <m/>
+    <n v="34"/>
+    <n v="9"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="3"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <n v="1"/>
+    <n v="2"/>
+    <n v="1"/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="4"/>
+    <n v="23"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="4"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="17"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="5"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="8"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="11"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="5"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="5"/>
+    <n v="9"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="6"/>
+    <n v="15"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="15"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="4"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="14"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="14"/>
+    <n v="4"/>
+    <n v="3"/>
+    <n v="5"/>
+    <n v="2"/>
+    <n v="10"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="9"/>
+    <n v="6"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="4"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="10"/>
+    <n v="5"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="7"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="11"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="3"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="12"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="3"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="13"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="4"/>
+    <m/>
+    <n v="4"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="24"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="14"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="15"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="16"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="17"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="3"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="18"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="19"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="20"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="6"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="21"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="9"/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="6"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="22"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="23"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="24"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="18"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="25"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="26"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="28"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="27"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="5"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="7"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="28"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="29"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="3"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="30"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="31"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="32"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="33"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="34"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <x v="14"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="2"/>
+  </r>
+  <r>
+    <x v="35"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="36"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+  </r>
+  <r>
+    <x v="37"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <n v="1"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DBFE69D1-2D07-43AB-87BD-4DC7DF1B4E10}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="25">
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="39">
+        <item x="26"/>
+        <item x="31"/>
+        <item x="25"/>
+        <item x="24"/>
+        <item x="19"/>
+        <item x="29"/>
+        <item x="4"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="30"/>
+        <item x="16"/>
+        <item x="1"/>
+        <item x="15"/>
+        <item x="34"/>
+        <item x="32"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item x="18"/>
+        <item x="7"/>
+        <item x="21"/>
+        <item x="9"/>
+        <item x="35"/>
+        <item x="33"/>
+        <item x="8"/>
+        <item x="5"/>
+        <item x="20"/>
+        <item x="37"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="2"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="14"/>
+        <item x="36"/>
+        <item x="0"/>
+        <item x="28"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="39">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Species" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3965,6 +5436,377 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A51440-23BC-4F33-82CE-E6A8A8A00B9E}">
+  <dimension ref="A3:B42"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="10" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B7" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B12" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B18" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B25" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B26" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B27" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B28" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B29" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="B30" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B34" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B37" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B38" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B39" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B41" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" s="9">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559A7446-AC0E-4CF9-B3DF-6897D0F8BD3D}">
   <dimension ref="A1:AW129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5036,7 +6878,9 @@
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
       <c r="X15" s="2"/>
-      <c r="Y15" s="2"/>
+      <c r="Y15" s="2">
+        <v>1</v>
+      </c>
       <c r="Z15" s="2"/>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
@@ -6682,7 +8526,7 @@
     </row>
     <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>109</v>
+        <v>167</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -6734,61 +8578,6 @@
       <c r="AU45" s="2"/>
       <c r="AV45" s="2"/>
       <c r="AW45" s="2"/>
-    </row>
-    <row r="46" spans="1:49" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="R46" s="2"/>
-      <c r="S46" s="2"/>
-      <c r="T46" s="2"/>
-      <c r="U46" s="2"/>
-      <c r="V46" s="2"/>
-      <c r="W46" s="2"/>
-      <c r="X46" s="2"/>
-      <c r="Y46" s="2">
-        <v>1</v>
-      </c>
-      <c r="Z46" s="2"/>
-      <c r="AA46" s="2"/>
-      <c r="AB46" s="2"/>
-      <c r="AC46" s="2"/>
-      <c r="AD46" s="2"/>
-      <c r="AE46" s="2"/>
-      <c r="AF46" s="2"/>
-      <c r="AG46" s="2"/>
-      <c r="AH46" s="2"/>
-      <c r="AI46" s="2"/>
-      <c r="AJ46" s="2"/>
-      <c r="AK46" s="2"/>
-      <c r="AL46" s="2"/>
-      <c r="AM46" s="2"/>
-      <c r="AN46" s="2"/>
-      <c r="AO46" s="2"/>
-      <c r="AP46" s="2"/>
-      <c r="AQ46" s="2"/>
-      <c r="AR46" s="2"/>
-      <c r="AS46" s="2"/>
-      <c r="AT46" s="2"/>
-      <c r="AU46" s="2"/>
-      <c r="AV46" s="2"/>
-      <c r="AW46" s="2"/>
     </row>
     <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
@@ -9560,7 +11349,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EC48DC0-45BD-4D9F-904E-3E6219ACF302}">
   <dimension ref="A1:AW72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -14212,7 +16001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{034E3BDA-6C7C-4827-8561-FE6C9D8E7C57}">
   <dimension ref="A1:E49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>